<commit_message>
fix: 'AW' added as 'E48'; currency in XML format with two decimal places
</commit_message>
<xml_diff>
--- a/TestRechnung.xlsx
+++ b/TestRechnung.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\herbe\Documents\Development\excel2zugferd\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E01B8AB-C28E-4BE6-A572-0DB0C9D462E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1019B041-5AD1-4ACC-8323-8A9218EF025B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="816" windowWidth="18348" windowHeight="13992" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15460" yWindow="2080" windowWidth="18540" windowHeight="11600" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -28,12 +28,15 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="39">
   <si>
     <t>An:</t>
   </si>
@@ -144,6 +147,12 @@
   </si>
   <si>
     <t>Das Datum für die Rechnung; Es wird nach "Rechnungsdatum:" gesucht.</t>
+  </si>
+  <si>
+    <t>Programmiertätigkeiten</t>
+  </si>
+  <si>
+    <t>AW</t>
   </si>
 </sst>
 </file>
@@ -572,22 +581,22 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:G15"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.109375" customWidth="1"/>
+    <col min="1" max="1" width="15.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -595,7 +604,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>35</v>
       </c>
@@ -603,7 +612,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>2</v>
       </c>
@@ -626,12 +635,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="F13" s="12" t="s">
         <v>8</v>
       </c>
@@ -639,7 +648,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="F14" s="12" t="s">
         <v>25</v>
       </c>
@@ -647,7 +656,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="F15" s="12" t="s">
         <v>11</v>
       </c>
@@ -667,43 +676,43 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:G38"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="24.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="53.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.5546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="13.5546875" style="10" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.6328125" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.08984375" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="53.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.54296875" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="13.54296875" style="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="7" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="7" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>1</v>
       </c>
@@ -711,7 +720,7 @@
         <v>20240001</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
         <v>33</v>
       </c>
@@ -722,8 +731,8 @@
         <v>34</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="10" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="10" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>2</v>
       </c>
@@ -746,7 +755,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="6">
         <v>1</v>
       </c>
@@ -763,15 +772,15 @@
         <v>9</v>
       </c>
       <c r="F11" s="12">
-        <f t="shared" ref="F11:F21" si="0">IF(E11="10 Min.",22,75)</f>
+        <f t="shared" ref="F11:F22" si="0">IF(E11="10 Min.",22,75)</f>
         <v>22</v>
       </c>
       <c r="G11" s="12">
-        <f t="shared" ref="G11:G21" si="1">D11*F11</f>
-        <v>22</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+        <f t="shared" ref="G11:G22" si="1">D11*F11</f>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="6">
         <f t="shared" ref="A12:A20" si="2">A11+1</f>
         <v>2</v>
@@ -797,7 +806,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="6">
         <f t="shared" si="2"/>
         <v>3</v>
@@ -823,7 +832,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="6">
         <f t="shared" si="2"/>
         <v>4</v>
@@ -849,7 +858,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="6">
         <f t="shared" si="2"/>
         <v>5</v>
@@ -875,7 +884,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="6">
         <f t="shared" si="2"/>
         <v>6</v>
@@ -901,7 +910,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="6">
         <f t="shared" si="2"/>
         <v>7</v>
@@ -927,7 +936,7 @@
         <v>525</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="6">
         <f t="shared" si="2"/>
         <v>8</v>
@@ -953,7 +962,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="6">
         <f t="shared" si="2"/>
         <v>9</v>
@@ -979,7 +988,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="6">
         <f t="shared" si="2"/>
         <v>10</v>
@@ -1005,7 +1014,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="3">
         <v>11</v>
       </c>
@@ -1027,86 +1036,106 @@
         <v>37.5</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E22" s="8"/>
-      <c r="F22" s="12"/>
-    </row>
-    <row r="23" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="3">
+        <v>12</v>
+      </c>
+      <c r="B22" s="2">
+        <v>45309</v>
+      </c>
+      <c r="C22" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D22" s="3">
+        <v>5</v>
+      </c>
+      <c r="E22" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F22" s="12">
+        <v>22</v>
+      </c>
+      <c r="G22" s="10">
+        <f t="shared" si="1"/>
+        <v>110</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E23" s="8"/>
       <c r="F23" s="12"/>
     </row>
-    <row r="24" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E24" s="8"/>
       <c r="F24" s="12"/>
     </row>
-    <row r="25" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E25" s="8"/>
       <c r="F25" s="12"/>
     </row>
-    <row r="26" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E26" s="8"/>
       <c r="F26" s="12"/>
     </row>
-    <row r="27" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E27" s="8"/>
       <c r="F27" s="12"/>
     </row>
-    <row r="28" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E28" s="8"/>
       <c r="F28" s="12"/>
     </row>
-    <row r="29" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E29" s="8"/>
       <c r="F29" s="12"/>
     </row>
-    <row r="30" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E30" s="8"/>
       <c r="F30" s="12"/>
     </row>
-    <row r="31" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E31" s="8"/>
       <c r="F31" s="12"/>
     </row>
-    <row r="32" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E32" s="8"/>
       <c r="F32" s="12"/>
     </row>
-    <row r="33" spans="5:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="5:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E33" s="8"/>
       <c r="F33" s="12"/>
     </row>
-    <row r="34" spans="5:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="5:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E34" s="8"/>
       <c r="F34" s="12"/>
     </row>
-    <row r="35" spans="5:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="5:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="F35" s="12" t="s">
         <v>8</v>
       </c>
       <c r="G35" s="12">
         <f>SUM(G11:G27)</f>
-        <v>994.5</v>
-      </c>
-    </row>
-    <row r="36" spans="5:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+        <v>1104.5</v>
+      </c>
+    </row>
+    <row r="36" spans="5:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="F36" s="12" t="s">
         <v>25</v>
       </c>
       <c r="G36" s="18">
         <f>G35*19%</f>
-        <v>188.95500000000001</v>
-      </c>
-    </row>
-    <row r="37" spans="5:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+        <v>209.85499999999999</v>
+      </c>
+    </row>
+    <row r="37" spans="5:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="F37" s="12" t="s">
         <v>11</v>
       </c>
       <c r="G37" s="18">
         <f>SUM(G35:G36)</f>
-        <v>1183.4549999999999</v>
-      </c>
-    </row>
-    <row r="38" spans="5:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+        <v>1314.355</v>
+      </c>
+    </row>
+    <row r="38" spans="5:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E38" s="8"/>
       <c r="F38" s="12"/>
     </row>
@@ -1119,43 +1148,43 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F435B499-96C6-4725-AFFC-8DE837C76B55}">
   <dimension ref="A1:G37"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="24.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="53.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.5546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="13.5546875" style="10" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.6328125" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.08984375" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="53.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.54296875" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="13.54296875" style="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="7" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="7" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>1</v>
       </c>
@@ -1163,8 +1192,8 @@
         <v>20240001</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="9" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="9" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>2</v>
       </c>
@@ -1187,7 +1216,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="6">
         <v>1</v>
       </c>
@@ -1212,7 +1241,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="6">
         <f t="shared" ref="A11:A19" si="2">A10+1</f>
         <v>2</v>
@@ -1238,7 +1267,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="6">
         <f t="shared" si="2"/>
         <v>3</v>
@@ -1264,7 +1293,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="6">
         <f t="shared" si="2"/>
         <v>4</v>
@@ -1290,7 +1319,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="6">
         <f t="shared" si="2"/>
         <v>5</v>
@@ -1316,7 +1345,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="6">
         <f t="shared" si="2"/>
         <v>6</v>
@@ -1342,7 +1371,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="6">
         <f t="shared" si="2"/>
         <v>7</v>
@@ -1368,7 +1397,7 @@
         <v>525</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="6">
         <f t="shared" si="2"/>
         <v>8</v>
@@ -1394,7 +1423,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="6">
         <f t="shared" si="2"/>
         <v>9</v>
@@ -1420,7 +1449,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="6">
         <f t="shared" si="2"/>
         <v>10</v>
@@ -1446,63 +1475,63 @@
         <v>22</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E20" s="8"/>
       <c r="F20" s="12"/>
     </row>
-    <row r="21" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E21" s="8"/>
       <c r="F21" s="12"/>
     </row>
-    <row r="22" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E22" s="8"/>
       <c r="F22" s="12"/>
     </row>
-    <row r="23" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E23" s="8"/>
       <c r="F23" s="12"/>
     </row>
-    <row r="24" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E24" s="8"/>
       <c r="F24" s="12"/>
     </row>
-    <row r="25" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E25" s="8"/>
       <c r="F25" s="12"/>
     </row>
-    <row r="26" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E26" s="8"/>
       <c r="F26" s="12"/>
     </row>
-    <row r="27" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E27" s="8"/>
       <c r="F27" s="12"/>
     </row>
-    <row r="28" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E28" s="8"/>
       <c r="F28" s="12"/>
     </row>
-    <row r="29" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E29" s="8"/>
       <c r="F29" s="12"/>
     </row>
-    <row r="30" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E30" s="8"/>
       <c r="F30" s="12"/>
     </row>
-    <row r="31" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E31" s="8"/>
       <c r="F31" s="12"/>
     </row>
-    <row r="32" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E32" s="8"/>
       <c r="F32" s="12"/>
     </row>
-    <row r="33" spans="5:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="5:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E33" s="8"/>
       <c r="F33" s="12"/>
     </row>
-    <row r="34" spans="5:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="5:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="F34" s="12" t="s">
         <v>8</v>
       </c>
@@ -1511,7 +1540,7 @@
         <v>957</v>
       </c>
     </row>
-    <row r="35" spans="5:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="5:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="F35" s="12" t="s">
         <v>25</v>
       </c>
@@ -1519,7 +1548,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="5:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="5:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="F36" s="12" t="s">
         <v>11</v>
       </c>
@@ -1528,7 +1557,7 @@
         <v>957</v>
       </c>
     </row>
-    <row r="37" spans="5:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="5:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E37" s="8"/>
       <c r="F37" s="12"/>
     </row>

</xml_diff>

<commit_message>
fix: tests corrected for added line in excel sheet
</commit_message>
<xml_diff>
--- a/TestRechnung.xlsx
+++ b/TestRechnung.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\herbe\Documents\Development\excel2zugferd\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1019B041-5AD1-4ACC-8323-8A9218EF025B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D1239C2-22F3-467E-86FF-29011CB26FC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15460" yWindow="2080" windowWidth="18540" windowHeight="11600" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-560" yWindow="870" windowWidth="18540" windowHeight="11600" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -228,7 +228,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -273,6 +273,9 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="44" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -772,7 +775,7 @@
         <v>9</v>
       </c>
       <c r="F11" s="12">
-        <f t="shared" ref="F11:F22" si="0">IF(E11="10 Min.",22,75)</f>
+        <f t="shared" ref="F11:F21" si="0">IF(E11="10 Min.",22,75)</f>
         <v>22</v>
       </c>
       <c r="G11" s="12">
@@ -1040,7 +1043,7 @@
       <c r="A22" s="3">
         <v>12</v>
       </c>
-      <c r="B22" s="2">
+      <c r="B22" s="19">
         <v>45309</v>
       </c>
       <c r="C22" s="16" t="s">

</xml_diff>

<commit_message>
feat: #33 different tax values possible
</commit_message>
<xml_diff>
--- a/TestRechnung.xlsx
+++ b/TestRechnung.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\herbe\Documents\Development\excel2zugferd\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D1239C2-22F3-467E-86FF-29011CB26FC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54692782-E704-46EF-B482-D0120FD5E291}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-560" yWindow="870" windowWidth="18540" windowHeight="11600" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1320" yWindow="530" windowWidth="26500" windowHeight="13130" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
     <sheet name="Rechnung2" sheetId="2" r:id="rId2"/>
     <sheet name="Rechnung für Kleinunternehmen" sheetId="3" r:id="rId3"/>
+    <sheet name="Rechnung div. Steuern" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="49">
   <si>
     <t>An:</t>
   </si>
@@ -153,6 +154,37 @@
   </si>
   <si>
     <t>AW</t>
+  </si>
+  <si>
+    <t>Steuer</t>
+  </si>
+  <si>
+    <t>Taxifahrt</t>
+  </si>
+  <si>
+    <t>Anfahrt dazu per Taxi</t>
+  </si>
+  <si>
+    <t>Umsatzsteueraufschlüsselung:</t>
+  </si>
+  <si>
+    <t>Umsatzsteuer</t>
+  </si>
+  <si>
+    <t>TÜV</t>
+  </si>
+  <si>
+    <t>Durchlaufender Posten im Sinne von § 10 Abs. 1 Satz 6 UStG</t>
+  </si>
+  <si>
+    <t>Steuerfreie Bildungsleistung gemäß § 4 Nr. 21 UStG</t>
+  </si>
+  <si>
+    <t>Stk.</t>
+  </si>
+  <si>
+    <t>Achtung: nur ein Typ einer Position mit Steuer 0,00% ist je Rechnung erlaubt.
+Hier widerspricht sich die Vorgabe mit den Prüfroutinen.</t>
   </si>
 </sst>
 </file>
@@ -163,7 +195,7 @@
     <numFmt numFmtId="44" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -199,6 +231,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -228,7 +267,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -276,6 +315,32 @@
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="1" xfId="1" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="4" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1567,4 +1632,534 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1156111F-A04F-4E96-8331-110DBD50F257}">
+  <dimension ref="A1:H38"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="24.6328125" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.08984375" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="53.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.54296875" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="13.54296875" style="10" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="7" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B7" s="13">
+        <v>20240001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B8" s="7">
+        <v>45321</v>
+      </c>
+      <c r="C8" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="10" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="F10" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="G10" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="H10" s="14" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="6">
+        <v>1</v>
+      </c>
+      <c r="B11" s="7">
+        <v>45292</v>
+      </c>
+      <c r="C11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D11" s="6">
+        <v>1</v>
+      </c>
+      <c r="E11" t="s">
+        <v>9</v>
+      </c>
+      <c r="F11" s="12">
+        <f t="shared" ref="F11:F19" si="0">IF(E11="10 Min.",22,75)</f>
+        <v>22</v>
+      </c>
+      <c r="G11" s="12">
+        <f t="shared" ref="G11:G21" si="1">D11*F11</f>
+        <v>22</v>
+      </c>
+      <c r="H11" s="23"/>
+    </row>
+    <row r="12" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="6">
+        <f t="shared" ref="A12:A21" si="2">A11+1</f>
+        <v>2</v>
+      </c>
+      <c r="B12" s="7">
+        <v>45293</v>
+      </c>
+      <c r="C12" t="s">
+        <v>17</v>
+      </c>
+      <c r="D12" s="6">
+        <v>1</v>
+      </c>
+      <c r="E12" t="s">
+        <v>9</v>
+      </c>
+      <c r="F12" s="12">
+        <f t="shared" si="0"/>
+        <v>22</v>
+      </c>
+      <c r="G12" s="12">
+        <f t="shared" si="1"/>
+        <v>22</v>
+      </c>
+      <c r="H12" s="23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="6">
+        <f t="shared" si="2"/>
+        <v>3</v>
+      </c>
+      <c r="B13" s="7">
+        <v>45294</v>
+      </c>
+      <c r="C13" t="s">
+        <v>40</v>
+      </c>
+      <c r="D13" s="6">
+        <v>1</v>
+      </c>
+      <c r="E13" t="s">
+        <v>47</v>
+      </c>
+      <c r="F13" s="12">
+        <v>55</v>
+      </c>
+      <c r="G13" s="12">
+        <f t="shared" si="1"/>
+        <v>55</v>
+      </c>
+      <c r="H13" s="23">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="6">
+        <f t="shared" si="2"/>
+        <v>4</v>
+      </c>
+      <c r="B14" s="7">
+        <v>45294</v>
+      </c>
+      <c r="C14" t="s">
+        <v>18</v>
+      </c>
+      <c r="D14" s="6">
+        <v>2</v>
+      </c>
+      <c r="E14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F14" s="12">
+        <f t="shared" si="0"/>
+        <v>75</v>
+      </c>
+      <c r="G14" s="12">
+        <f t="shared" si="1"/>
+        <v>150</v>
+      </c>
+      <c r="H14" s="23"/>
+    </row>
+    <row r="15" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="6">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="B15" s="7">
+        <v>45295</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D15" s="6">
+        <v>1</v>
+      </c>
+      <c r="E15" t="s">
+        <v>9</v>
+      </c>
+      <c r="F15" s="12">
+        <f t="shared" si="0"/>
+        <v>22</v>
+      </c>
+      <c r="G15" s="12">
+        <f t="shared" si="1"/>
+        <v>22</v>
+      </c>
+      <c r="H15" s="23"/>
+    </row>
+    <row r="16" spans="1:8" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="6">
+        <f t="shared" si="2"/>
+        <v>6</v>
+      </c>
+      <c r="B16" s="7">
+        <v>45296</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="D16" s="6">
+        <v>1</v>
+      </c>
+      <c r="E16" t="s">
+        <v>10</v>
+      </c>
+      <c r="F16" s="12">
+        <f t="shared" si="0"/>
+        <v>75</v>
+      </c>
+      <c r="G16" s="12">
+        <f t="shared" si="1"/>
+        <v>75</v>
+      </c>
+      <c r="H16" s="23"/>
+    </row>
+    <row r="17" spans="1:8" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="6">
+        <f t="shared" si="2"/>
+        <v>7</v>
+      </c>
+      <c r="B17" s="7">
+        <v>45302</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D17" s="6">
+        <v>7</v>
+      </c>
+      <c r="E17" t="s">
+        <v>10</v>
+      </c>
+      <c r="F17" s="12">
+        <f t="shared" si="0"/>
+        <v>75</v>
+      </c>
+      <c r="G17" s="12">
+        <f t="shared" si="1"/>
+        <v>525</v>
+      </c>
+      <c r="H17" s="23"/>
+    </row>
+    <row r="18" spans="1:8" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="6">
+        <f t="shared" si="2"/>
+        <v>8</v>
+      </c>
+      <c r="B18" s="7">
+        <v>45302</v>
+      </c>
+      <c r="C18" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="D18" s="6">
+        <v>1</v>
+      </c>
+      <c r="E18" t="s">
+        <v>47</v>
+      </c>
+      <c r="F18" s="12">
+        <v>130</v>
+      </c>
+      <c r="G18" s="12">
+        <f t="shared" si="1"/>
+        <v>130</v>
+      </c>
+      <c r="H18" s="23">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="6">
+        <f t="shared" si="2"/>
+        <v>9</v>
+      </c>
+      <c r="B19" s="7">
+        <v>45309</v>
+      </c>
+      <c r="C19" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D19" s="6">
+        <v>1</v>
+      </c>
+      <c r="E19" t="s">
+        <v>10</v>
+      </c>
+      <c r="F19" s="12">
+        <f t="shared" si="0"/>
+        <v>75</v>
+      </c>
+      <c r="G19" s="12">
+        <f t="shared" si="1"/>
+        <v>75</v>
+      </c>
+      <c r="H19" s="23"/>
+    </row>
+    <row r="20" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="6">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="B20" s="7"/>
+      <c r="C20" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="D20" s="20">
+        <v>1</v>
+      </c>
+      <c r="E20" s="28" t="s">
+        <v>47</v>
+      </c>
+      <c r="F20" s="12">
+        <v>96</v>
+      </c>
+      <c r="G20" s="10">
+        <f t="shared" si="1"/>
+        <v>96</v>
+      </c>
+      <c r="H20" s="23">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="6">
+        <f t="shared" si="2"/>
+        <v>11</v>
+      </c>
+      <c r="B21" s="19">
+        <v>45309</v>
+      </c>
+      <c r="C21" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D21" s="3">
+        <v>5</v>
+      </c>
+      <c r="E21" s="28" t="s">
+        <v>38</v>
+      </c>
+      <c r="F21" s="12">
+        <v>22</v>
+      </c>
+      <c r="G21" s="10">
+        <f t="shared" si="1"/>
+        <v>110</v>
+      </c>
+      <c r="H21" s="23"/>
+    </row>
+    <row r="22" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="6"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="12"/>
+      <c r="H22" s="23"/>
+    </row>
+    <row r="23" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="6"/>
+      <c r="E23" s="8"/>
+      <c r="F23" s="12"/>
+      <c r="H23" s="23"/>
+    </row>
+    <row r="24" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="6"/>
+      <c r="E24" s="8"/>
+      <c r="F24" s="12"/>
+      <c r="H24" s="23"/>
+    </row>
+    <row r="25" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E25" s="8"/>
+      <c r="F25" s="12"/>
+      <c r="H25" s="23"/>
+    </row>
+    <row r="26" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E26" s="8"/>
+      <c r="F26" s="12"/>
+      <c r="H26" s="23"/>
+    </row>
+    <row r="27" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E27" s="8"/>
+      <c r="F27" s="12"/>
+    </row>
+    <row r="28" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E28" s="27" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E29" s="25">
+        <v>1</v>
+      </c>
+      <c r="F29" s="24">
+        <v>0.19</v>
+      </c>
+      <c r="G29" s="10">
+        <f>SUMIFS(G11:G26,H11:H26,"")+SUMIFS(G11:G26,H11:H26,E29)</f>
+        <v>1001</v>
+      </c>
+      <c r="H29" s="21">
+        <f>G29*F29</f>
+        <v>190.19</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E30" s="25">
+        <v>2</v>
+      </c>
+      <c r="F30" s="24">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="G30" s="10">
+        <f>SUMIFS(G11:G26,H11:H26,E30)</f>
+        <v>151</v>
+      </c>
+      <c r="H30" s="21">
+        <f>G30*F30</f>
+        <v>10.57</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E31" s="26">
+        <v>3</v>
+      </c>
+      <c r="F31" s="24">
+        <v>0</v>
+      </c>
+      <c r="G31" s="10">
+        <f>SUMIFS(G11:G26,H11:H26,E31)</f>
+        <v>130</v>
+      </c>
+      <c r="H31" s="22" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" ht="91" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="29" t="s">
+        <v>48</v>
+      </c>
+      <c r="E32" s="26">
+        <v>4</v>
+      </c>
+      <c r="F32" s="24">
+        <v>0</v>
+      </c>
+      <c r="G32" s="10">
+        <f>SUMIFS(G12:G27,H12:H27,E32)</f>
+        <v>0</v>
+      </c>
+      <c r="H32" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="33" spans="5:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E33" s="8"/>
+      <c r="F33" s="12"/>
+    </row>
+    <row r="34" spans="5:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E34" s="8"/>
+      <c r="F34" s="12"/>
+    </row>
+    <row r="35" spans="5:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="F35" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="G35" s="12">
+        <f>SUM(G11:G26)</f>
+        <v>1282</v>
+      </c>
+    </row>
+    <row r="36" spans="5:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="F36" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="G36" s="18">
+        <f>SUM(H29:H33)</f>
+        <v>200.76</v>
+      </c>
+    </row>
+    <row r="37" spans="5:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="F37" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="G37" s="18">
+        <f>SUM(G35:G36)</f>
+        <v>1482.76</v>
+      </c>
+    </row>
+    <row r="38" spans="5:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E38" s="8"/>
+      <c r="F38" s="12"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix: allow multiple different types of tax free items in one bill
</commit_message>
<xml_diff>
--- a/TestRechnung.xlsx
+++ b/TestRechnung.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\herbe\Documents\Development\excel2zugferd\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54692782-E704-46EF-B482-D0120FD5E291}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF7C14C4-8BB5-4EBE-A07A-E92FAD41FD3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1320" yWindow="530" windowWidth="26500" windowHeight="13130" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="49">
   <si>
     <t>An:</t>
   </si>
@@ -183,8 +183,7 @@
     <t>Stk.</t>
   </si>
   <si>
-    <t>Achtung: nur ein Typ einer Position mit Steuer 0,00% ist je Rechnung erlaubt.
-Hier widerspricht sich die Vorgabe mit den Prüfroutinen.</t>
+    <t>Schulung VHS Kurs</t>
   </si>
 </sst>
 </file>
@@ -1636,7 +1635,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1156111F-A04F-4E96-8331-110DBD50F257}">
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="24.6328125" style="3" bestFit="1" customWidth="1"/>
@@ -1736,18 +1735,18 @@
         <v>9</v>
       </c>
       <c r="F11" s="12">
-        <f t="shared" ref="F11:F19" si="0">IF(E11="10 Min.",22,75)</f>
+        <f t="shared" ref="F11:F20" si="0">IF(E11="10 Min.",22,75)</f>
         <v>22</v>
       </c>
       <c r="G11" s="12">
-        <f t="shared" ref="G11:G21" si="1">D11*F11</f>
+        <f t="shared" ref="G11:G22" si="1">D11*F11</f>
         <v>22</v>
       </c>
       <c r="H11" s="23"/>
     </row>
     <row r="12" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="6">
-        <f t="shared" ref="A12:A21" si="2">A11+1</f>
+        <f t="shared" ref="A12:A22" si="2">A11+1</f>
         <v>2</v>
       </c>
       <c r="B12" s="7">
@@ -1811,7 +1810,7 @@
         <v>45294</v>
       </c>
       <c r="C14" t="s">
-        <v>18</v>
+        <v>48</v>
       </c>
       <c r="D14" s="6">
         <v>2</v>
@@ -1827,7 +1826,9 @@
         <f t="shared" si="1"/>
         <v>150</v>
       </c>
-      <c r="H14" s="23"/>
+      <c r="H14" s="23">
+        <v>4</v>
+      </c>
     </row>
     <row r="15" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="6">
@@ -1838,23 +1839,25 @@
         <v>45295</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>19</v>
+        <v>48</v>
       </c>
       <c r="D15" s="6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E15" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F15" s="12">
         <f t="shared" si="0"/>
-        <v>22</v>
+        <v>75</v>
       </c>
       <c r="G15" s="12">
         <f t="shared" si="1"/>
-        <v>22</v>
-      </c>
-      <c r="H15" s="23"/>
+        <v>150</v>
+      </c>
+      <c r="H15" s="23">
+        <v>4</v>
+      </c>
     </row>
     <row r="16" spans="1:8" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="6">
@@ -1865,10 +1868,10 @@
         <v>45296</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>20</v>
+        <v>48</v>
       </c>
       <c r="D16" s="6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E16" t="s">
         <v>10</v>
@@ -1879,9 +1882,11 @@
       </c>
       <c r="G16" s="12">
         <f t="shared" si="1"/>
-        <v>75</v>
-      </c>
-      <c r="H16" s="23"/>
+        <v>150</v>
+      </c>
+      <c r="H16" s="23">
+        <v>4</v>
+      </c>
     </row>
     <row r="17" spans="1:8" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="6">
@@ -1892,10 +1897,10 @@
         <v>45302</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>21</v>
+        <v>48</v>
       </c>
       <c r="D17" s="6">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E17" t="s">
         <v>10</v>
@@ -1906,9 +1911,11 @@
       </c>
       <c r="G17" s="12">
         <f t="shared" si="1"/>
-        <v>525</v>
-      </c>
-      <c r="H17" s="23"/>
+        <v>150</v>
+      </c>
+      <c r="H17" s="23">
+        <v>4</v>
+      </c>
     </row>
     <row r="18" spans="1:8" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="6">
@@ -1944,7 +1951,7 @@
         <v>9</v>
       </c>
       <c r="B19" s="7">
-        <v>45309</v>
+        <v>45308</v>
       </c>
       <c r="C19" s="9" t="s">
         <v>23</v>
@@ -1965,30 +1972,33 @@
       </c>
       <c r="H19" s="23"/>
     </row>
-    <row r="20" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="6">
         <f t="shared" si="2"/>
         <v>10</v>
       </c>
-      <c r="B20" s="7"/>
-      <c r="C20" s="16" t="s">
-        <v>41</v>
-      </c>
-      <c r="D20" s="20">
-        <v>1</v>
-      </c>
-      <c r="E20" s="28" t="s">
-        <v>47</v>
+      <c r="B20" s="7">
+        <v>45309</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="D20" s="6">
+        <v>2</v>
+      </c>
+      <c r="E20" t="s">
+        <v>10</v>
       </c>
       <c r="F20" s="12">
-        <v>96</v>
-      </c>
-      <c r="G20" s="10">
-        <f t="shared" si="1"/>
-        <v>96</v>
+        <f t="shared" si="0"/>
+        <v>75</v>
+      </c>
+      <c r="G20" s="12">
+        <f t="shared" si="1"/>
+        <v>150</v>
       </c>
       <c r="H20" s="23">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -1996,31 +2006,51 @@
         <f t="shared" si="2"/>
         <v>11</v>
       </c>
-      <c r="B21" s="19">
+      <c r="B21" s="7"/>
+      <c r="C21" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="D21" s="20">
+        <v>1</v>
+      </c>
+      <c r="E21" s="28" t="s">
+        <v>47</v>
+      </c>
+      <c r="F21" s="12">
+        <v>96</v>
+      </c>
+      <c r="G21" s="10">
+        <f t="shared" si="1"/>
+        <v>96</v>
+      </c>
+      <c r="H21" s="23">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="6">
+        <f t="shared" si="2"/>
+        <v>12</v>
+      </c>
+      <c r="B22" s="19">
         <v>45309</v>
       </c>
-      <c r="C21" s="16" t="s">
+      <c r="C22" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="D21" s="3">
+      <c r="D22" s="3">
         <v>5</v>
       </c>
-      <c r="E21" s="28" t="s">
+      <c r="E22" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="F21" s="12">
-        <v>22</v>
-      </c>
-      <c r="G21" s="10">
+      <c r="F22" s="12">
+        <v>22</v>
+      </c>
+      <c r="G22" s="10">
         <f t="shared" si="1"/>
         <v>110</v>
       </c>
-      <c r="H21" s="23"/>
-    </row>
-    <row r="22" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="6"/>
-      <c r="E22" s="8"/>
-      <c r="F22" s="12"/>
       <c r="H22" s="23"/>
     </row>
     <row r="23" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -2036,6 +2066,7 @@
       <c r="H24" s="23"/>
     </row>
     <row r="25" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="6"/>
       <c r="E25" s="8"/>
       <c r="F25" s="12"/>
       <c r="H25" s="23"/>
@@ -2048,115 +2079,118 @@
     <row r="27" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E27" s="8"/>
       <c r="F27" s="12"/>
+      <c r="H27" s="23"/>
     </row>
     <row r="28" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="E28" s="27" t="s">
+      <c r="E28" s="8"/>
+      <c r="F28" s="12"/>
+    </row>
+    <row r="29" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E29" s="27" t="s">
         <v>42</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="E29" s="25">
-        <v>1</v>
-      </c>
-      <c r="F29" s="24">
-        <v>0.19</v>
-      </c>
-      <c r="G29" s="10">
-        <f>SUMIFS(G11:G26,H11:H26,"")+SUMIFS(G11:G26,H11:H26,E29)</f>
-        <v>1001</v>
-      </c>
-      <c r="H29" s="21">
-        <f>G29*F29</f>
-        <v>190.19</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E30" s="25">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F30" s="24">
-        <v>7.0000000000000007E-2</v>
+        <v>0.19</v>
       </c>
       <c r="G30" s="10">
-        <f>SUMIFS(G11:G26,H11:H26,E30)</f>
-        <v>151</v>
+        <f>SUMIFS(G11:G27,H11:H27,"")+SUMIFS(G11:G27,H11:H27,E30)</f>
+        <v>229</v>
       </c>
       <c r="H30" s="21">
         <f>G30*F30</f>
+        <v>43.51</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E31" s="25">
+        <v>2</v>
+      </c>
+      <c r="F31" s="24">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="G31" s="10">
+        <f>SUMIFS(G11:G27,H11:H27,E31)</f>
+        <v>151</v>
+      </c>
+      <c r="H31" s="21">
+        <f>G31*F31</f>
         <v>10.57</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="E31" s="26">
+    <row r="32" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E32" s="26">
         <v>3</v>
-      </c>
-      <c r="F31" s="24">
-        <v>0</v>
-      </c>
-      <c r="G31" s="10">
-        <f>SUMIFS(G11:G26,H11:H26,E31)</f>
-        <v>130</v>
-      </c>
-      <c r="H31" s="22" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" ht="91" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="29" t="s">
-        <v>48</v>
-      </c>
-      <c r="E32" s="26">
-        <v>4</v>
       </c>
       <c r="F32" s="24">
         <v>0</v>
       </c>
       <c r="G32" s="10">
-        <f>SUMIFS(G12:G27,H12:H27,E32)</f>
+        <f>SUMIFS(G11:G27,H11:H27,E32)</f>
+        <v>130</v>
+      </c>
+      <c r="H32" s="22" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" ht="21.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="29"/>
+      <c r="E33" s="26">
+        <v>4</v>
+      </c>
+      <c r="F33" s="24">
         <v>0</v>
       </c>
-      <c r="H32" t="s">
+      <c r="G33" s="10">
+        <f>SUMIFS(G12:G28,H12:H28,E33)</f>
+        <v>750</v>
+      </c>
+      <c r="H33" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="33" spans="5:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="E33" s="8"/>
-      <c r="F33" s="12"/>
-    </row>
-    <row r="34" spans="5:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E34" s="8"/>
       <c r="F34" s="12"/>
     </row>
-    <row r="35" spans="5:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="F35" s="12" t="s">
+    <row r="35" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E35" s="8"/>
+      <c r="F35" s="12"/>
+    </row>
+    <row r="36" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="F36" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="G35" s="12">
-        <f>SUM(G11:G26)</f>
-        <v>1282</v>
-      </c>
-    </row>
-    <row r="36" spans="5:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="F36" s="12" t="s">
+      <c r="G36" s="12">
+        <f>SUM(G11:G27)</f>
+        <v>1260</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="F37" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="G36" s="18">
-        <f>SUM(H29:H33)</f>
-        <v>200.76</v>
-      </c>
-    </row>
-    <row r="37" spans="5:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="F37" s="12" t="s">
+      <c r="G37" s="18">
+        <f>SUM(H30:H34)</f>
+        <v>54.08</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="F38" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="G37" s="18">
-        <f>SUM(G35:G36)</f>
-        <v>1482.76</v>
-      </c>
-    </row>
-    <row r="38" spans="5:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="E38" s="8"/>
-      <c r="F38" s="12"/>
+      <c r="G38" s="18">
+        <f>SUM(G36:G37)</f>
+        <v>1314.08</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E39" s="8"/>
+      <c r="F39" s="12"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix: extended fault tolerance
</commit_message>
<xml_diff>
--- a/TestRechnung.xlsx
+++ b/TestRechnung.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\herbe\Documents\Development\excel2zugferd\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF7C14C4-8BB5-4EBE-A07A-E92FAD41FD3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BCE834C5-1DD3-40F6-9FA2-F04941D92C9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1320" yWindow="530" windowWidth="26500" windowHeight="13130" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6930" yWindow="550" windowWidth="26500" windowHeight="13130" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>

</xml_diff>